<commit_message>
Update soccer trades 2026-08-10 00:02:57 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
+++ b/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
+          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -542,12 +542,12 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>331.57222</t>
+          <t>128</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.7988</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786316229</t>
+          <t>1786316612</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>415.11389</t>
+          <t>160.0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
+          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -646,12 +646,12 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>20.70997</t>
+          <t>256</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786316213</t>
+          <t>1786316590</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>26.009381</t>
+          <t>320.0</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,92 +739,84 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
+          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>331.57222</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.7988</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>74.68</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1.3613</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>L19066036</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786310047</t>
+          <t>1786316229</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -834,7 +826,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>206.726644</t>
+          <t>415.11389</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,92 +843,84 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
+          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>20.70997</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.7963</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>65.17485</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>1.745</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>L19066036</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786309443</t>
+          <t>1786316213</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +930,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>87.48302</t>
+          <t>26.009381</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,7 +947,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -978,22 +962,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>39.22</t>
+          <t>74.68</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.1575</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1018,7 +1002,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1048,7 +1032,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786294983</t>
+          <t>1786310047</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>249.015873</t>
+          <t>206.726644</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,36 +1059,44 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>105.38217</t>
+          <t>65.17485</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
@@ -1122,7 +1114,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1144,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786309443</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1154,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>374.69216</t>
+          <t>87.48302</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,7 +1171,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1194,47 +1186,47 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>72.13</t>
+          <t>39.22</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2112</t>
+          <t>1.1575</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (4)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1264,7 +1256,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786294983</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1274,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>341.443787</t>
+          <t>249.015873</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,110 +1283,326 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>105.38217</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.2812</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>374.69216</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>72.13</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.2112</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>341.443787</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>0x3694b34366b9210385b305bea639feafe31d2c1f0ae196fbd04597fed8e17499</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>1.5463</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>L19066036</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>1786234530</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>1786561200</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>1.830664</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-10 10:02:37 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
+++ b/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
+          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.2163</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,7 +559,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -608,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786316612</t>
+          <t>1786334647</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>160.0</t>
+          <t>13.872832</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
+          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -646,7 +654,7 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>128</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -712,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786316590</t>
+          <t>1786316612</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -722,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>320.0</t>
+          <t>160.0</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
+          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -750,12 +758,12 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>331.57222</t>
+          <t>256</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.7988</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -816,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786316229</t>
+          <t>1786316590</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -826,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>415.11389</t>
+          <t>320.0</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,7 +851,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
+          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -854,12 +862,12 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>20.70997</t>
+          <t>331.57222</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.7988</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -920,7 +928,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786316213</t>
+          <t>1786316229</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -930,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>26.009381</t>
+          <t>415.11389</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -947,92 +955,84 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
+          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>20.70997</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.7963</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>74.68</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>1.3613</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>L19066036</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786310047</t>
+          <t>1786316213</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>206.726644</t>
+          <t>26.009381</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,12 +1059,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
+          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1074,22 +1074,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>65.17485</t>
+          <t>74.68</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786309443</t>
+          <t>1786310047</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>87.48302</t>
+          <t>206.726644</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1171,12 +1171,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1186,22 +1186,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>39.22</t>
+          <t>65.17485</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.1575</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786294983</t>
+          <t>1786309443</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>249.015873</t>
+          <t>87.48302</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,7 +1283,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1291,28 +1291,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>105.38217</t>
+          <t>39.22</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.1575</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
@@ -1330,7 +1338,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1360,7 +1368,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786294983</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1370,7 +1378,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>374.69216</t>
+          <t>249.015873</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1387,7 +1395,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1395,81 +1403,73 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>105.38217</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.2812</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>72.13</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>1.2112</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>L19066036</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R10" t="inlineStr">
         <is>
           <t>1786294922</t>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>341.443787</t>
+          <t>374.69216</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,110 +1499,222 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>72.13</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.2112</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>341.443787</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>0x3694b34366b9210385b305bea639feafe31d2c1f0ae196fbd04597fed8e17499</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>1.5463</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>L19066036</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>1786234530</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>1786561200</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>1.830664</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-10 20:02:26 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
+++ b/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:V15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
+          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,39 +546,39 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>12.49</t>
+          <t>13.13154</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5475</t>
+          <t>1.065</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Aston Villa</t>
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786371203</t>
+          <t>1786390904</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>22.812785</t>
+          <t>202.023692</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
+          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,47 +658,47 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11.30985</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.2163</t>
+          <t>1.065</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786334647</t>
+          <t>1786390902</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>13.872832</t>
+          <t>173.997692</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,23 +755,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
+          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>12.49</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.5475</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -779,7 +783,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -802,7 +810,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786316612</t>
+          <t>1786371203</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>160.0</t>
+          <t>22.812785</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,23 +867,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
+          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.2163</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -883,7 +895,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -936,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786316590</t>
+          <t>1786334647</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>320.0</t>
+          <t>13.872832</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
+          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -974,12 +990,12 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>331.57222</t>
+          <t>128</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.7988</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1040,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786316229</t>
+          <t>1786316612</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1050,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>415.11389</t>
+          <t>160.0</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,7 +1083,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
+          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1078,12 +1094,12 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>20.70997</t>
+          <t>256</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1144,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786316213</t>
+          <t>1786316590</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1154,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>26.009381</t>
+          <t>320.0</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1171,39 +1187,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
+          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>74.68</t>
+          <t>331.57222</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.3613</t>
+          <t>1.7988</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1226,7 +1234,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1256,7 +1264,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786310047</t>
+          <t>1786316229</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1266,7 +1274,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>206.726644</t>
+          <t>415.11389</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,39 +1291,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
+          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>65.17485</t>
+          <t>20.70997</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.7963</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786309443</t>
+          <t>1786316213</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>87.48302</t>
+          <t>26.009381</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1410,22 +1410,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>39.22</t>
+          <t>74.68</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.1575</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786294983</t>
+          <t>1786310047</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>249.015873</t>
+          <t>206.726644</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,36 +1507,44 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>105.38217</t>
+          <t>65.17485</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
@@ -1554,7 +1562,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1584,7 +1592,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786309443</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1594,7 +1602,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>374.69216</t>
+          <t>87.48302</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1611,7 +1619,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1626,47 +1634,47 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>72.13</t>
+          <t>39.22</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.2112</t>
+          <t>1.1575</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (4)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1696,7 +1704,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786294983</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1706,7 +1714,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>341.443787</t>
+          <t>249.015873</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1723,110 +1731,326 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>105.38217</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.2812</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>374.69216</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>72.13</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.2112</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>341.443787</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>0x3694b34366b9210385b305bea639feafe31d2c1f0ae196fbd04597fed8e17499</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>1.5463</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>L19066036</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
         <is>
           <t>1786234530</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>1786561200</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>1.830664</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 01:02:46 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
+++ b/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
+          <t>0xd637b84dae82a7f4481771e1d20283f17db1805dd930164e9bb8dbed3a2b9b48</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>13.13154</t>
+          <t>216.99999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.065</t>
+          <t>1.4888</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Over 5.0</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -586,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786390904</t>
+          <t>1786409895</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>202.023692</t>
+          <t>443.989749</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
+          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,7 +650,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11.30985</t>
+          <t>13.13154</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -728,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786390902</t>
+          <t>1786390904</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>173.997692</t>
+          <t>202.023692</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +747,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
+          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,39 +762,39 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>12.49</t>
+          <t>11.30985</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5475</t>
+          <t>1.065</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>Aston Villa</t>
@@ -810,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786371203</t>
+          <t>1786390902</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>22.812785</t>
+          <t>173.997692</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,12 +859,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
+          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -882,12 +874,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12.49</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.2163</t>
+          <t>1.5475</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -897,32 +889,32 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -952,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786334647</t>
+          <t>1786371203</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +954,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>13.872832</t>
+          <t>22.812785</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,23 +971,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
+          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.2163</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1003,7 +999,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786316612</t>
+          <t>1786334647</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>160.0</t>
+          <t>13.872832</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,7 +1083,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
+          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1094,7 +1094,7 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>128</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786316590</t>
+          <t>1786316612</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>320.0</t>
+          <t>160.0</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
+          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1198,12 +1198,12 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>331.57222</t>
+          <t>256</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.7988</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786316229</t>
+          <t>1786316590</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>415.11389</t>
+          <t>320.0</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,7 +1291,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
+          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1302,12 +1302,12 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>20.70997</t>
+          <t>331.57222</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.7988</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786316213</t>
+          <t>1786316229</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>26.009381</t>
+          <t>415.11389</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,39 +1395,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
+          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>74.68</t>
+          <t>20.70997</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.3613</t>
+          <t>1.7963</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1450,7 +1442,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1480,7 +1472,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786310047</t>
+          <t>1786316213</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1490,7 +1482,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>206.726644</t>
+          <t>26.009381</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,12 +1499,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
+          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1522,22 +1514,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>65.17485</t>
+          <t>74.68</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1562,7 +1554,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1592,7 +1584,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786309443</t>
+          <t>1786310047</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1602,7 +1594,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>87.48302</t>
+          <t>206.726644</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,12 +1611,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1634,22 +1626,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>39.22</t>
+          <t>65.17485</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.1575</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1674,7 +1666,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1704,7 +1696,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786294983</t>
+          <t>1786309443</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1714,7 +1706,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>249.015873</t>
+          <t>87.48302</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,7 +1723,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1739,28 +1731,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>105.38217</t>
+          <t>39.22</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.1575</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786294983</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>374.69216</t>
+          <t>249.015873</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1835,7 +1835,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1843,54 +1843,46 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>72.13</t>
+          <t>105.38217</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2112</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1930,7 +1922,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>341.443787</t>
+          <t>374.69216</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,110 +1939,222 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>72.13</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.2112</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>341.443787</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>0x3694b34366b9210385b305bea639feafe31d2c1f0ae196fbd04597fed8e17499</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>1.5463</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>L19066036</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
         <is>
           <t>1786234530</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>1786561200</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>1.830664</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 05:02:43 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
+++ b/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xd637b84dae82a7f4481771e1d20283f17db1805dd930164e9bb8dbed3a2b9b48</t>
+          <t>0x0116fe81833bb6a4ed2dbacecc0bf888c42afc5f3f40bf376cb5bbc37cb8d843</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -542,12 +542,12 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>216.99999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4888</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786409895</t>
+          <t>1786421953</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>443.989749</t>
+          <t>2.040816</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,39 +635,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
+          <t>0x8cc01473b0041a94127de7aaaa3c878a17f610392cc876d414055d273a76d3ab</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>13.13154</t>
+          <t>68</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.065</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Over 5.0</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -690,7 +682,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786390904</t>
+          <t>1786421917</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>202.023692</t>
+          <t>138.77551</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,39 +739,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
+          <t>0x5aa13b0d414124958cbfe600c479d7f26d1e6a5f24ed35b4d6a600eb47503f89</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>11.30985</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.065</t>
+          <t>1.4888</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Over 5.0</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -802,7 +786,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +816,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786390902</t>
+          <t>1786421886</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +826,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>173.997692</t>
+          <t>18.414322</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,54 +843,46 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
+          <t>0xd637b84dae82a7f4481771e1d20283f17db1805dd930164e9bb8dbed3a2b9b48</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>12.49</t>
+          <t>216.99999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.5475</t>
+          <t>1.4888</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>Aston Villa</t>
@@ -914,7 +890,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +920,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786371203</t>
+          <t>1786409895</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +930,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>22.812785</t>
+          <t>443.989749</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,12 +947,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
+          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -986,47 +962,47 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13.13154</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.2163</t>
+          <t>1.065</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1056,7 +1032,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786334647</t>
+          <t>1786390904</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>13.872832</t>
+          <t>202.023692</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,31 +1059,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
+          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>11.30985</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.065</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1130,7 +1114,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1160,7 +1144,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786316612</t>
+          <t>1786390902</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1154,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>160.0</t>
+          <t>173.997692</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,23 +1171,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
+          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>12.49</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.5475</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1211,7 +1199,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1234,7 +1226,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1264,7 +1256,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786316590</t>
+          <t>1786371203</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1274,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>320.0</t>
+          <t>22.812785</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,23 +1283,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
+          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>331.57222</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.7988</t>
+          <t>1.2163</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1315,7 +1311,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786316229</t>
+          <t>1786334647</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>415.11389</t>
+          <t>13.872832</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
+          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1406,12 +1406,12 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>20.70997</t>
+          <t>128</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786316213</t>
+          <t>1786316612</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>26.009381</t>
+          <t>160.0</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,39 +1499,31 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
+          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>74.68</t>
+          <t>256</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.3613</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1554,7 +1546,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1584,7 +1576,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786310047</t>
+          <t>1786316590</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1594,7 +1586,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>206.726644</t>
+          <t>320.0</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1611,39 +1603,31 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
+          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>65.17485</t>
+          <t>331.57222</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.7988</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1666,7 +1650,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1696,7 +1680,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786309443</t>
+          <t>1786316229</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1706,7 +1690,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>87.48302</t>
+          <t>415.11389</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1723,39 +1707,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>39.22</t>
+          <t>20.70997</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.1575</t>
+          <t>1.7963</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Over 4.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1778,7 +1754,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1808,7 +1784,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786294983</t>
+          <t>1786316213</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1818,7 +1794,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>249.015873</t>
+          <t>26.009381</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1835,7 +1811,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1843,28 +1819,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>105.38217</t>
+          <t>74.68</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
@@ -1882,7 +1866,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1912,7 +1896,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786310047</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1922,7 +1906,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>374.69216</t>
+          <t>206.726644</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1939,12 +1923,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1954,47 +1938,47 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>72.13</t>
+          <t>65.17485</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.2112</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2024,7 +2008,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786309443</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2034,7 +2018,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>341.443787</t>
+          <t>87.48302</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,110 +2035,438 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>39.22</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.1575</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1786294983</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>249.015873</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>105.38217</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.2812</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>374.69216</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>72.13</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.2112</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>341.443787</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>0x3694b34366b9210385b305bea639feafe31d2c1f0ae196fbd04597fed8e17499</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>1.5463</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>L19066036</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
         <is>
           <t>1786234530</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>1786561200</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>1.830664</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 06:02:30 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
+++ b/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,31 +531,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x0116fe81833bb6a4ed2dbacecc0bf888c42afc5f3f40bf376cb5bbc37cb8d843</t>
+          <t>0x62018a330ac2dc1528134a0e9913f5615e54c162ca453b2e278133061bd850c5</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6.00999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.5475</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -578,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786421953</t>
+          <t>1786424623</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2.040816</t>
+          <t>10.977151</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x8cc01473b0041a94127de7aaaa3c878a17f610392cc876d414055d273a76d3ab</t>
+          <t>0x0116fe81833bb6a4ed2dbacecc0bf888c42afc5f3f40bf376cb5bbc37cb8d843</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -646,7 +654,7 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -712,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786421917</t>
+          <t>1786421953</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -722,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>138.77551</t>
+          <t>2.040816</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x5aa13b0d414124958cbfe600c479d7f26d1e6a5f24ed35b4d6a600eb47503f89</t>
+          <t>0x8cc01473b0041a94127de7aaaa3c878a17f610392cc876d414055d273a76d3ab</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -750,12 +758,12 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>68</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4888</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -816,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786421886</t>
+          <t>1786421917</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -826,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>18.414322</t>
+          <t>138.77551</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,7 +851,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xd637b84dae82a7f4481771e1d20283f17db1805dd930164e9bb8dbed3a2b9b48</t>
+          <t>0x5aa13b0d414124958cbfe600c479d7f26d1e6a5f24ed35b4d6a600eb47503f89</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -854,7 +862,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>216.99999</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -920,7 +928,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786409895</t>
+          <t>1786421886</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -930,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>443.989749</t>
+          <t>18.414322</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -947,39 +955,31 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
+          <t>0xd637b84dae82a7f4481771e1d20283f17db1805dd930164e9bb8dbed3a2b9b48</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>13.13154</t>
+          <t>216.99999</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.065</t>
+          <t>1.4888</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Over 5.0</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786390904</t>
+          <t>1786409895</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>202.023692</t>
+          <t>443.989749</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,7 +1059,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
+          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>11.30985</t>
+          <t>13.13154</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786390902</t>
+          <t>1786390904</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>173.997692</t>
+          <t>202.023692</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1171,12 +1171,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
+          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1186,39 +1186,39 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>12.49</t>
+          <t>11.30985</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5475</t>
+          <t>1.065</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>Aston Villa</t>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786371203</t>
+          <t>1786390902</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>22.812785</t>
+          <t>173.997692</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,12 +1283,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
+          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12.49</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.2163</t>
+          <t>1.5475</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1313,32 +1313,32 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786334647</t>
+          <t>1786371203</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>13.872832</t>
+          <t>22.812785</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,23 +1395,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
+          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.2163</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1419,7 +1423,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1472,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786316612</t>
+          <t>1786334647</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1482,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>160.0</t>
+          <t>13.872832</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,7 +1507,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
+          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1510,7 +1518,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>128</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1576,7 +1584,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786316590</t>
+          <t>1786316612</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1586,7 +1594,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>320.0</t>
+          <t>160.0</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1603,7 +1611,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
+          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1614,12 +1622,12 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>331.57222</t>
+          <t>256</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.7988</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1680,7 +1688,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786316229</t>
+          <t>1786316590</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1690,7 +1698,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>415.11389</t>
+          <t>320.0</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1707,7 +1715,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
+          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1718,12 +1726,12 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>20.70997</t>
+          <t>331.57222</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.7988</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1784,7 +1792,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786316213</t>
+          <t>1786316229</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1794,7 +1802,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>26.009381</t>
+          <t>415.11389</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1811,39 +1819,31 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
+          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>74.68</t>
+          <t>20.70997</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.3613</t>
+          <t>1.7963</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1866,7 +1866,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786310047</t>
+          <t>1786316213</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>206.726644</t>
+          <t>26.009381</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1923,12 +1923,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
+          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1938,22 +1938,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>65.17485</t>
+          <t>74.68</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786309443</t>
+          <t>1786310047</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>87.48302</t>
+          <t>206.726644</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2035,12 +2035,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2050,22 +2050,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>39.22</t>
+          <t>65.17485</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.1575</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786294983</t>
+          <t>1786309443</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>249.015873</t>
+          <t>87.48302</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2155,28 +2155,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>105.38217</t>
+          <t>39.22</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.1575</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
@@ -2194,7 +2202,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2224,7 +2232,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786294983</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2234,7 +2242,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>374.69216</t>
+          <t>249.015873</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2251,7 +2259,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2259,54 +2267,46 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>72.13</t>
+          <t>105.38217</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.2112</t>
+          <t>1.2812</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>341.443787</t>
+          <t>374.69216</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2363,110 +2363,222 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>72.13</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.2112</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>341.443787</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>0x3694b34366b9210385b305bea639feafe31d2c1f0ae196fbd04597fed8e17499</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>1.5463</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>L19066036</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
         <is>
           <t>1786234530</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>1786561200</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>1.830664</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="V20" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 18:03:13 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
+++ b/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V26"/>
+  <dimension ref="A1:V29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xf05a004202d5172597115d20ed24213b9155c5d6fd7480d1fcb926574d5bb930</t>
+          <t>0xacfbb4991bf5c10a0276eaf4ab838401611edc56dc36a00f64cbacc0b4aaf142</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -542,17 +542,17 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>11.21</t>
+          <t>42.52</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x1ff093a0d6aad6ea34f9661babedbc7a361e7167b1f31f3dab05f34988e51f47</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786462484</t>
+          <t>1786466862</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>24.911111</t>
+          <t>586.482759</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,62 +635,54 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x9cd0218c04dbf9f8af03b16eef0d1cb40183eedfc941b885be7072ccb0f6a775</t>
+          <t>0xa4e38c77c1133d8be3d4c471cd270781599d373bbf4f6633ea6c2682fde48a52</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xe6a674A10b8bA44d086Cf85791B188209a1F6e2c</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>23.9188</t>
+          <t>9.88</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.215</t>
+          <t>1.5925</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0x67230bcb83f942bc217c5d745ea1712885e0906db6bd151cb38c9c1c8672117b</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786460921</t>
+          <t>1786466015</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>111.250233</t>
+          <t>16.675105</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,31 +739,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x315b979409334c6c5a235b8d158f0209e5839bd2f05831b53a9a292c608ee337</t>
+          <t>0x0da0312ac7181e4204b626031b1afcd3e2858ddc869ad4c77e972506b878493f</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>119.23</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.6187</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -794,7 +794,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786459823</t>
+          <t>1786465613</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>3.232323</t>
+          <t>662.388889</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,28 +851,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x44ab0a6adaab9b2b3e75e30bce10bd9f61fcccddc98d090614d9f0cfb8d3e00d</t>
+          <t>0xf05a004202d5172597115d20ed24213b9155c5d6fd7480d1fcb926574d5bb930</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>11.21</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -898,7 +898,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786459704</t>
+          <t>1786462484</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>343.089431</t>
+          <t>24.911111</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,31 +955,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xcdcdc100ea2811013be002432e70309f4738884853ece5cc8cd335e1b4ab4d0b</t>
+          <t>0x9cd0218c04dbf9f8af03b16eef0d1cb40183eedfc941b885be7072ccb0f6a775</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xF77AceaD3B354FCD16E60e4a6AbEdB7796b7094E</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0xe6a674A10b8bA44d086Cf85791B188209a1F6e2c</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>280.99999</t>
+          <t>23.9188</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.215</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1002,7 +1010,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1032,7 +1040,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786459347</t>
+          <t>1786460921</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1042,7 +1050,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>456.910553</t>
+          <t>111.250233</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,28 +1067,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x391ce88d76018af43c090050bc3937faecb44a3bb6876c2eb020f0d4a40fecb6</t>
+          <t>0x315b979409334c6c5a235b8d158f0209e5839bd2f05831b53a9a292c608ee337</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>312.25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4825</t>
+          <t>1.6187</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1106,7 +1114,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1136,7 +1144,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786431942</t>
+          <t>1786459823</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1146,7 +1154,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>647.150259</t>
+          <t>3.232323</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1163,54 +1171,46 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x62018a330ac2dc1528134a0e9913f5615e54c162ca453b2e278133061bd850c5</t>
+          <t>0x44ab0a6adaab9b2b3e75e30bce10bd9f61fcccddc98d090614d9f0cfb8d3e00d</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>6.00999</t>
+          <t>211</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5475</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>Aston Villa</t>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786424623</t>
+          <t>1786459704</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>10.977151</t>
+          <t>343.089431</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1275,28 +1275,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x0116fe81833bb6a4ed2dbacecc0bf888c42afc5f3f40bf376cb5bbc37cb8d843</t>
+          <t>0xcdcdc100ea2811013be002432e70309f4738884853ece5cc8cd335e1b4ab4d0b</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+          <t>0xF77AceaD3B354FCD16E60e4a6AbEdB7796b7094E</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>280.99999</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.615</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786421953</t>
+          <t>1786459347</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2.040816</t>
+          <t>456.910553</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1379,23 +1379,23 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x8cc01473b0041a94127de7aaaa3c878a17f610392cc876d414055d273a76d3ab</t>
+          <t>0x391ce88d76018af43c090050bc3937faecb44a3bb6876c2eb020f0d4a40fecb6</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>312.25</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.4825</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786421917</t>
+          <t>1786431942</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>138.77551</t>
+          <t>647.150259</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1483,31 +1483,39 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x5aa13b0d414124958cbfe600c479d7f26d1e6a5f24ed35b4d6a600eb47503f89</t>
+          <t>0x62018a330ac2dc1528134a0e9913f5615e54c162ca453b2e278133061bd850c5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6.00999</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.4888</t>
+          <t>1.5475</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1530,7 +1538,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1560,7 +1568,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786421886</t>
+          <t>1786424623</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1570,7 +1578,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>18.414322</t>
+          <t>10.977151</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1587,7 +1595,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xd637b84dae82a7f4481771e1d20283f17db1805dd930164e9bb8dbed3a2b9b48</t>
+          <t>0x0116fe81833bb6a4ed2dbacecc0bf888c42afc5f3f40bf376cb5bbc37cb8d843</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1598,12 +1606,12 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>216.99999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.4888</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1664,7 +1672,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786409895</t>
+          <t>1786421953</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1674,7 +1682,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>443.989749</t>
+          <t>2.040816</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1691,39 +1699,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
+          <t>0x8cc01473b0041a94127de7aaaa3c878a17f610392cc876d414055d273a76d3ab</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13.13154</t>
+          <t>68</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.065</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Over 5.0</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786390904</t>
+          <t>1786421917</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>202.023692</t>
+          <t>138.77551</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1803,39 +1803,31 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
+          <t>0x5aa13b0d414124958cbfe600c479d7f26d1e6a5f24ed35b4d6a600eb47503f89</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11.30985</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.065</t>
+          <t>1.4888</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Over 5.0</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1858,7 +1850,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1888,7 +1880,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786390902</t>
+          <t>1786421886</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1898,7 +1890,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>173.997692</t>
+          <t>18.414322</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1915,54 +1907,46 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
+          <t>0xd637b84dae82a7f4481771e1d20283f17db1805dd930164e9bb8dbed3a2b9b48</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>12.49</t>
+          <t>216.99999</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.5475</t>
+          <t>1.4888</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>Aston Villa</t>
@@ -1970,7 +1954,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2000,7 +1984,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786371203</t>
+          <t>1786409895</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2010,7 +1994,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>22.812785</t>
+          <t>443.989749</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2027,12 +2011,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
+          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2042,47 +2026,47 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13.13154</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.2163</t>
+          <t>1.065</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2112,7 +2096,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786334647</t>
+          <t>1786390904</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2122,7 +2106,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>13.872832</t>
+          <t>202.023692</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2139,31 +2123,39 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
+          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>11.30985</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.065</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -2186,7 +2178,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2216,7 +2208,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786316612</t>
+          <t>1786390902</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2226,7 +2218,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>160.0</t>
+          <t>173.997692</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2243,23 +2235,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
+          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>12.49</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.5475</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2267,7 +2263,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786316590</t>
+          <t>1786371203</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>320.0</t>
+          <t>22.812785</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2347,23 +2347,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
+          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>331.57222</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.7988</t>
+          <t>1.2163</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2371,7 +2375,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -2424,7 +2432,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786316229</t>
+          <t>1786334647</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2434,7 +2442,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>415.11389</t>
+          <t>13.872832</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2451,7 +2459,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
+          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2462,12 +2470,12 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>20.70997</t>
+          <t>128</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2528,7 +2536,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786316213</t>
+          <t>1786316612</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2538,7 +2546,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>26.009381</t>
+          <t>160.0</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2555,39 +2563,31 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
+          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>74.68</t>
+          <t>256</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.3613</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -2610,7 +2610,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786310047</t>
+          <t>1786316590</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>206.726644</t>
+          <t>320.0</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2667,39 +2667,31 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
+          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>65.17485</t>
+          <t>331.57222</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.7988</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -2722,7 +2714,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2752,7 +2744,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786309443</t>
+          <t>1786316229</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2762,7 +2754,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>87.48302</t>
+          <t>415.11389</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2779,39 +2771,31 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>39.22</t>
+          <t>20.70997</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.1575</t>
+          <t>1.7963</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Over 4.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -2834,7 +2818,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2864,7 +2848,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786294983</t>
+          <t>1786316213</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2874,7 +2858,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>249.015873</t>
+          <t>26.009381</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2891,7 +2875,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2899,28 +2883,36 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>105.38217</t>
+          <t>74.68</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.3613</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
@@ -2938,7 +2930,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2968,7 +2960,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786310047</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2978,7 +2970,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>374.69216</t>
+          <t>206.726644</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2995,12 +2987,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3010,47 +3002,47 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>72.13</t>
+          <t>65.17485</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.2112</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3080,7 +3072,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786309443</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3090,7 +3082,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>341.443787</t>
+          <t>87.48302</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3107,110 +3099,438 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>39.22</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.1575</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1786294983</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>249.015873</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>105.38217</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.2812</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>374.69216</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>72.13</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.2112</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>341.443787</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>0x3694b34366b9210385b305bea639feafe31d2c1f0ae196fbd04597fed8e17499</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>1.5463</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>L19066036</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
         <is>
           <t>1786234530</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="S29" t="inlineStr">
         <is>
           <t>1786561200</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>1.830664</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr">
+      <c r="V29" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-12 00:02:51 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
+++ b/data/sxbet/ligas/UEFA Super Cup/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V34"/>
+  <dimension ref="A1:V56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xb1f0749faa19666cf4234a512073b6fe905a80f4e19d7462647cfe9ceb57c06d</t>
+          <t>0x5e9b92a3ee864ed306ae19b1eb8415371da432df1801adf9df4096158c2ada97</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.94</t>
+          <t>22.15226</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.4475</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -586,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
+          <t>0x633e1f4af7bf294be4c13c5c783beb3d10adbea62e87950389cb3cfa326086cb</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786477844</t>
+          <t>1786491019</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>44.882051</t>
+          <t>49.502257</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,31 +635,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xe75fd64786bddcffb26a2ab8aec8ff02c007fcc64ee16062ab2bed40a67d164f</t>
+          <t>0x23733dbdf9fa3729981e360673c4b7d7c10ff2531e371c5badad3796d6c9c512</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x85Da26Dce2e5F76FcFb411d89ceb8fcf11A9CBcD</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>27.55999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4487</t>
+          <t>1.5575</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain -0.5</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -690,7 +690,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x633e1f4af7bf294be4c13c5c783beb3d10adbea62e87950389cb3cfa326086cb</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786477225</t>
+          <t>1786490560</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>6016.713092</t>
+          <t>49.43496</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,23 +747,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x3c9edc4f5c44c0dbcf413728ce35f4f8c68b50f2abbeb2caa42a72a09516164e</t>
+          <t>0x0727088f0a4a30c10d202e7c81d28be4eb0ab98bf21e981e558f2e5179605bac</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xa498150823d867380b25175554a275c1c668256e</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>688.37615</t>
+          <t>15.81921</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4487</t>
+          <t>1.4463</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786476767</t>
+          <t>1786490214</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1533.98585</t>
+          <t>35.44921</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,7 +851,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x951615130443e4362647a81545c8c088c7317365c4ffa9a07467321ade98f125</t>
+          <t>0x2e03fcc3f7ecc087552ed1d69a1f8008e36e398bfe42ea205ce282f08f1c1340</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -866,12 +866,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>17.97</t>
+          <t>13.87999</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.2437</t>
+          <t>1.5562</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Paris Saint Germain</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786476263</t>
+          <t>1786490114</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>73.723077</t>
+          <t>24.952791</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,12 +963,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x14d842428ba2fc42cb9122fcef1e8ea4d521ff5e928fa03d4027a9e9d36cce69</t>
+          <t>0x031e42fbfd08a3c7d769259edbc4291e998075aee0ff949b46b2ff5a320f4fb9</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -978,12 +978,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.3075</t>
+          <t>1.3062</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786473059</t>
+          <t>1786487872</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>15.447154</t>
+          <t>3.62449</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,31 +1075,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xacfbb4991bf5c10a0276eaf4ab838401611edc56dc36a00f64cbacc0b4aaf142</t>
+          <t>0x973ce82e34197c696686774e4b32dc293666e3b1f344b3c042ea8e0bc0baf472</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>42.52</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.0725</t>
+          <t>1.2463</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1122,7 +1130,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x1ff093a0d6aad6ea34f9661babedbc7a361e7167b1f31f3dab05f34988e51f47</t>
+          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786466862</t>
+          <t>1786484906</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>586.482759</t>
+          <t>12.182741</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,31 +1187,39 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xa4e38c77c1133d8be3d4c471cd270781599d373bbf4f6633ea6c2682fde48a52</t>
+          <t>0x4189c1704e3efda1c32f863bee5edac536cbbc1ddc5c7ff92ffcec3f8671f4dd</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>9.88</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5925</t>
+          <t>1.53</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1226,7 +1242,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x67230bcb83f942bc217c5d745ea1712885e0906db6bd151cb38c9c1c8672117b</t>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1256,7 +1272,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786466015</t>
+          <t>1786483830</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1266,7 +1282,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>16.675105</t>
+          <t>9.433962</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,7 +1299,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x0da0312ac7181e4204b626031b1afcd3e2858ddc869ad4c77e972506b878493f</t>
+          <t>0x86035074a77352f25945be3c07a1ce0a72476812a4d9ee7a5d31accc0005ca8e</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1298,22 +1314,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>119.23</t>
+          <t>2.14549</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.5275</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1338,7 +1354,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1368,7 +1384,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786465613</t>
+          <t>1786483821</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1378,7 +1394,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>662.388889</t>
+          <t>4.06728</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,28 +1411,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xf05a004202d5172597115d20ed24213b9155c5d6fd7480d1fcb926574d5bb930</t>
+          <t>0x95d1a72bec5f6cbef6a0bee578fc49d11315543f98d64986bc30ab10b98ab235</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x64f5b1770dC9BeAdAA5c573F52472842f8894c8C</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>11.21</t>
+          <t>300</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>1.6987</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1442,7 +1458,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x409d8b258d8921e8f4a2c11460cbb794c2d8610abb209e4090e8a8ae8f39d2d7</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1472,7 +1488,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786462484</t>
+          <t>1786481014</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1482,7 +1498,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>24.911111</t>
+          <t>429.338104</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,62 +1515,54 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x9cd0218c04dbf9f8af03b16eef0d1cb40183eedfc941b885be7072ccb0f6a775</t>
+          <t>0x75abf2cc9245d94d8697557465991a972b17d428172f9c86e5103ccf4513ae1d</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xe6a674A10b8bA44d086Cf85791B188209a1F6e2c</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>23.9188</t>
+          <t>280.65999</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.215</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0x409d8b258d8921e8f4a2c11460cbb794c2d8610abb209e4090e8a8ae8f39d2d7</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1584,7 +1592,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786460921</t>
+          <t>1786479821</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1594,7 +1602,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>111.250233</t>
+          <t>400.942843</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1611,31 +1619,39 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x315b979409334c6c5a235b8d158f0209e5839bd2f05831b53a9a292c608ee337</t>
+          <t>0x7b6931100ecd01485a88a37e39d7604129b6c1b4774ef01d18474422b8022991</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>295.34</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.6187</t>
+          <t>1.2437</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1658,7 +1674,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1688,7 +1704,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786459823</t>
+          <t>1786479008</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1698,7 +1714,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>3.232323</t>
+          <t>1211.651282</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1715,28 +1731,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x44ab0a6adaab9b2b3e75e30bce10bd9f61fcccddc98d090614d9f0cfb8d3e00d</t>
+          <t>0xfd5730799b860d55deb75e792b32577fe97b21a6872bcdcae76b7d727aa3f5e1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
+          <t>0xa498150823d867380b25175554a275c1c668256e</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>15.78675</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.445</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1762,7 +1778,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1792,7 +1808,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786459704</t>
+          <t>1786478908</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1802,7 +1818,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>343.089431</t>
+          <t>35.475843</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1819,28 +1835,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xcdcdc100ea2811013be002432e70309f4738884853ece5cc8cd335e1b4ab4d0b</t>
+          <t>0xaa6b20356dec3ef3de3c3740df5cda0bfaf51ac484d1b2f78d6d001ebf63c609</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xF77AceaD3B354FCD16E60e4a6AbEdB7796b7094E</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>280.99999</t>
+          <t>0.00327</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.7675</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1866,7 +1882,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1896,7 +1912,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786459347</t>
+          <t>1786478826</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1906,7 +1922,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>456.910553</t>
+          <t>0.004261</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1923,7 +1939,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x391ce88d76018af43c090050bc3937faecb44a3bb6876c2eb020f0d4a40fecb6</t>
+          <t>0x1ca2c2e3faa5fd0586c76f29023f0ae32e5b7eb91a5e924bff0c79c1fd8e3978</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1931,23 +1947,31 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>312.25</t>
+          <t>7.61</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.4825</t>
+          <t>1.2437</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -1970,7 +1994,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2000,7 +2024,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786431942</t>
+          <t>1786478809</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2010,7 +2034,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>647.150259</t>
+          <t>31.220513</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2027,27 +2051,23 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x62018a330ac2dc1528134a0e9913f5615e54c162ca453b2e278133061bd850c5</t>
+          <t>0xd719c5ae636d9e747b1caa23c9df7ac916d22589ebafce09e6a90f528305ad43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6.00999</t>
+          <t>30.2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.5475</t>
+          <t>1.76</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2055,26 +2075,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>Aston Villa</t>
@@ -2082,7 +2098,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2112,7 +2128,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786424623</t>
+          <t>1786478807</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2122,7 +2138,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>10.977151</t>
+          <t>39.736842</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2139,31 +2155,39 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x0116fe81833bb6a4ed2dbacecc0bf888c42afc5f3f40bf376cb5bbc37cb8d843</t>
+          <t>0x7e152d80b0c185c0abe8c4ca426947b4261d81003670d3822de824587a968e1d</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>27.91</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.5637</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>Asian Handicap (-0.5)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain -0.5</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -2186,7 +2210,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+          <t>0x633e1f4af7bf294be4c13c5c783beb3d10adbea62e87950389cb3cfa326086cb</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2216,7 +2240,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786421953</t>
+          <t>1786478806</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2226,7 +2250,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2.040816</t>
+          <t>49.507761</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2243,31 +2267,39 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x8cc01473b0041a94127de7aaaa3c878a17f610392cc876d414055d273a76d3ab</t>
+          <t>0x762726fa569798e9bb38e6d1d3a6718a3e6b17854ec943996f440407d07d5af1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>30.51955</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.205</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -2290,7 +2322,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2320,7 +2352,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786421917</t>
+          <t>1786478801</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2330,7 +2362,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>138.77551</t>
+          <t>148.875854</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2347,31 +2379,39 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x5aa13b0d414124958cbfe600c479d7f26d1e6a5f24ed35b4d6a600eb47503f89</t>
+          <t>0x8e47fef69d97d7a182f242c2cdce1afab730128f4310cd28a6f9c5d37adae0d1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>36.47459</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.4888</t>
+          <t>1.245</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -2394,7 +2434,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2424,7 +2464,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786421886</t>
+          <t>1786478798</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2434,7 +2474,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>18.414322</t>
+          <t>148.875878</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2451,28 +2491,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xd637b84dae82a7f4481771e1d20283f17db1805dd930164e9bb8dbed3a2b9b48</t>
+          <t>0x4b13bf02996be9f8f2f945b0a566bfd6a4a430bd57ac43a76f92d64f15f5498d</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+          <t>0x0dc32f656f382cB67758F43c4d29A281feE11B76</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>216.99999</t>
+          <t>66.06366</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.4888</t>
+          <t>1.4438</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -2498,7 +2538,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2528,7 +2568,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786409895</t>
+          <t>1786478774</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2538,7 +2578,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>443.989749</t>
+          <t>148.875854</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2555,39 +2595,31 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
+          <t>0xe9e3237227be288d77eb896c110ca16fd4018525f8bcea0d1e30930f9032da8b</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>13.13154</t>
+          <t>2.10999</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.065</t>
+          <t>1.76</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Over 5.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -2610,7 +2642,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
+          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2640,7 +2672,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786390904</t>
+          <t>1786478768</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2650,7 +2682,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>202.023692</t>
+          <t>2.776303</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2667,12 +2699,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
+          <t>0x4c9eb0ce8768b1300644ee9d6d756f3477ae0a67da7b2d98350ea8c35a646255</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2682,22 +2714,22 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>11.30985</t>
+          <t>13.35</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.065</t>
+          <t>1.5613</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Over 5.0</t>
+          <t>Paris Saint Germain</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2722,7 +2754,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2752,7 +2784,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786390902</t>
+          <t>1786478575</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2762,7 +2794,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>173.997692</t>
+          <t>23.786192</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2779,27 +2811,23 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
+          <t>0x3991dd65a93f5a305e8899432f4bb1612f1b874d3aa09a9a9266778002ba1f22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>12.49</t>
+          <t>280.97998</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.5475</t>
+          <t>1.76</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2807,26 +2835,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
       <c r="K23" t="inlineStr">
         <is>
           <t>Aston Villa</t>
@@ -2834,7 +2858,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2864,7 +2888,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786371203</t>
+          <t>1786478575</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2874,7 +2898,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>22.812785</t>
+          <t>369.7105</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2891,12 +2915,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
+          <t>0xb1f0749faa19666cf4234a512073b6fe905a80f4e19d7462647cfe9ceb57c06d</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2906,12 +2930,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10.94</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.2163</t>
+          <t>1.2437</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2921,32 +2945,32 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>UEFA Super Cup</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain vs Aston Villa</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Paris Saint Germain</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Aston Villa</t>
-        </is>
-      </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2976,7 +3000,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786334647</t>
+          <t>1786477844</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2986,7 +3010,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>13.872832</t>
+          <t>44.882051</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3003,23 +3027,23 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
+          <t>0xe75fd64786bddcffb26a2ab8aec8ff02c007fcc64ee16062ab2bed40a67d164f</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x85Da26Dce2e5F76FcFb411d89ceb8fcf11A9CBcD</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.4487</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3050,7 +3074,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3080,7 +3104,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786316612</t>
+          <t>1786477225</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3090,7 +3114,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>160.0</t>
+          <t>6016.713092</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3107,23 +3131,23 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
+          <t>0x3c9edc4f5c44c0dbcf413728ce35f4f8c68b50f2abbeb2caa42a72a09516164e</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0xa498150823d867380b25175554a275c1c668256e</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>688.37615</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.4487</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3154,7 +3178,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3184,7 +3208,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786316590</t>
+          <t>1786476767</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3194,7 +3218,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>320.0</t>
+          <t>1533.98585</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3211,23 +3235,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
+          <t>0x951615130443e4362647a81545c8c088c7317365c4ffa9a07467321ade98f125</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>331.57222</t>
+          <t>17.97</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.7988</t>
+          <t>1.2437</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3235,7 +3263,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -3258,7 +3290,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0x82142b3963732a3fdd36aa8afa37f80a8be5d40f1cde3d8c81b2a40f833fd442</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3288,7 +3320,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786316229</t>
+          <t>1786476263</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3298,7 +3330,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>415.11389</t>
+          <t>73.723077</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3315,7 +3347,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
+          <t>0x14d842428ba2fc42cb9122fcef1e8ea4d521ff5e928fa03d4027a9e9d36cce69</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3323,23 +3355,31 @@
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>20.70997</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.7963</t>
+          <t>1.3075</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -3362,7 +3402,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+          <t>0x1eb0162b5ef5cce461102a0a0589d643a0342cf1c36981096646de6b5d6f255c</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3392,7 +3432,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786316213</t>
+          <t>1786473059</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3402,7 +3442,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>26.009381</t>
+          <t>15.447154</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3419,39 +3459,31 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
+          <t>0xacfbb4991bf5c10a0276eaf4ab838401611edc56dc36a00f64cbacc0b4aaf142</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>74.68</t>
+          <t>42.52</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.3613</t>
+          <t>1.0725</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -3474,7 +3506,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+          <t>0x1ff093a0d6aad6ea34f9661babedbc7a361e7167b1f31f3dab05f34988e51f47</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3504,7 +3536,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786310047</t>
+          <t>1786466862</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3514,7 +3546,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>206.726644</t>
+          <t>586.482759</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3531,39 +3563,31 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
+          <t>0xa4e38c77c1133d8be3d4c471cd270781599d373bbf4f6633ea6c2682fde48a52</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>65.17485</t>
+          <t>9.88</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.5925</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
@@ -3586,7 +3610,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
+          <t>0x67230bcb83f942bc217c5d745ea1712885e0906db6bd151cb38c9c1c8672117b</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3616,7 +3640,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786309443</t>
+          <t>1786466015</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3626,7 +3650,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>87.48302</t>
+          <t>16.675105</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3643,7 +3667,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+          <t>0x0da0312ac7181e4204b626031b1afcd3e2858ddc869ad4c77e972506b878493f</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3658,12 +3682,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>39.22</t>
+          <t>119.23</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.1575</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3728,7 +3752,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786294983</t>
+          <t>1786465613</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3738,7 +3762,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>249.015873</t>
+          <t>662.388889</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3755,28 +3779,28 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+          <t>0xf05a004202d5172597115d20ed24213b9155c5d6fd7480d1fcb926574d5bb930</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>105.38217</t>
+          <t>11.21</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.2812</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>UEFA Super Cup</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -3802,7 +3826,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3832,7 +3856,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786462484</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3842,7 +3866,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>374.69216</t>
+          <t>24.911111</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3859,12 +3883,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+          <t>0x9cd0218c04dbf9f8af03b16eef0d1cb40183eedfc941b885be7072ccb0f6a775</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xe6a674A10b8bA44d086Cf85791B188209a1F6e2c</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3874,12 +3898,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>72.13</t>
+          <t>23.9188</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.2112</t>
+          <t>1.215</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3944,7 +3968,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786294922</t>
+          <t>1786460921</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3954,7 +3978,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>341.443787</t>
+          <t>111.250233</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3971,110 +3995,2470 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>0x315b979409334c6c5a235b8d158f0209e5839bd2f05831b53a9a292c608ee337</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.6187</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>1786459823</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>3.232323</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>0x44ab0a6adaab9b2b3e75e30bce10bd9f61fcccddc98d090614d9f0cfb8d3e00d</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.615</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>1786459704</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>343.089431</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>0xcdcdc100ea2811013be002432e70309f4738884853ece5cc8cd335e1b4ab4d0b</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0xF77AceaD3B354FCD16E60e4a6AbEdB7796b7094E</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>280.99999</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1.615</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>1786459347</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>456.910553</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>0x391ce88d76018af43c090050bc3937faecb44a3bb6876c2eb020f0d4a40fecb6</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>312.25</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.4825</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>1786431942</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>647.150259</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>0x62018a330ac2dc1528134a0e9913f5615e54c162ca453b2e278133061bd850c5</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>6.00999</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.5475</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1786424623</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>10.977151</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>0x0116fe81833bb6a4ed2dbacecc0bf888c42afc5f3f40bf376cb5bbc37cb8d843</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>1786421953</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>2.040816</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>0x8cc01473b0041a94127de7aaaa3c878a17f610392cc876d414055d273a76d3ab</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>1786421917</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>138.77551</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>0x5aa13b0d414124958cbfe600c479d7f26d1e6a5f24ed35b4d6a600eb47503f89</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1.4888</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>1786421886</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>18.414322</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>0xd637b84dae82a7f4481771e1d20283f17db1805dd930164e9bb8dbed3a2b9b48</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0xDF62cAdd15F2cdB9b77E33884C759EE1cC7E6B6F</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>216.99999</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.4888</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>1786409895</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>443.989749</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>0x0ab7816a5b3bdeaa0ba243255d84fb7f5cc3010de74a12da7f4d57039736f910</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>13.13154</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1.065</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>1786390904</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>202.023692</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>0x3aecbb07f8e0603691063857af897a5688fe1c580e893e34227756577b554840</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>11.30985</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.065</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>0x05de8cf718f651bf384fc504b594eb03c576258ba7c4caaac4f5ff50201b6be3</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>1786390902</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>173.997692</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>0xc97d6568011afd75563e28f1a8282ebccaf6f6273338bd7d8803734afe501645</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>12.49</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1.5475</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>0xd90089ceb0c9854c3d68a3f09fc4fa855b3a26537e60e3a02b69256aaacd29db</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>1786371203</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>22.812785</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0xaf9559a19ef2d1861cd2330ba21b5fd736cd393bd5191bca5483f2fc312d54a0</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0x0C2DA7fC8702784d6f75c78Da25460783A6709a0</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.2163</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>1786334647</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>13.872832</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0x849efb290909a4a2724fa2fa8a31f1df72258e9472be51c9ba51d2240af02322</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>1786316612</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>160.0</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0x2b0477ef51d712b04d8ef50487a04f3c3c81ca210cfe2c567ba0f14a62c50675</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>1786316590</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>320.0</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0xe304d63b730df7947810a5d651289683a05fbd1b8bc83a59cf6e118f7145ff29</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>331.57222</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1.7988</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>1786316229</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>415.11389</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0xb37f867e7b09912283071b63d9f0d8dac6471b774c39329e6933acee2f2d4b67</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>20.70997</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1.7963</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>1786316213</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>26.009381</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0x85dd5b21bc7c1918df3fb950031e49fc0d13fd6e40115f33583a8beab3642acf</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>74.68</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>1.3613</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>0x1680a9183d7746c5c4672e850418adf866cefd179c8c9fa8a47ddd9aae14f195</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>1786310047</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>206.726644</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0xf090a9e8174708f430ff88479074f453c3c72df4065b04abe9083b733a2de742</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>0xE531A1CE55b94E311cC1629a6D68cAcf4F74d044</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>65.17485</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1.745</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>0xf1a8eb36f90ceb169cf77914181a6a20df69437e3abbd370109196ebd13c7edb</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>1786309443</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>87.48302</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0x98179b3dacaa2fd7ee4e1333c1e7254db907c541dd260df7fb7497696b21d6f3</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>39.22</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1.1575</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>0xcad766c3bece5254ba9d1a2b8cfdb650e513e674480798bb8979b1e953d44175</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>1786294983</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>249.015873</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0xf97a74664dd0407e7e5528292e63812f04a796ef7088678563661be1ae37038a</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>105.38217</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1.2812</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>0xe606a9a450716acc469c52d4cd4cc88af08c2e17027af860e1d62789a6948773</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>374.69216</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>0x74d74e84545efa9c898ad15f279d372ae4dcbbf0b95dd8b1d0652f6f472bd4c2</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>72.13</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>1.2112</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>UEFA Super Cup</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Paris Saint Germain</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>0x7d79a11368f71901641550937f2120d0c09dccfc84328fabe81c1eb7847ce4b5</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>L19066036</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>1786294922</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>1786561200</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>341.443787</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>0x3694b34366b9210385b305bea639feafe31d2c1f0ae196fbd04597fed8e17499</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>0x2B0D772143059220738CEC4818Ff2a1a499c48fD</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>1.5463</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>Under/Over (2.5)</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>Over 2.5</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H56" t="inlineStr">
         <is>
           <t>UEFA Super Cup</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>Paris Saint Germain vs Aston Villa</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J56" t="inlineStr">
         <is>
           <t>Paris Saint Germain</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>Aston Villa</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L56" t="inlineStr">
         <is>
           <t>0x40d2c11bb90148bb1491fd1a5f8f94c6aaefad0b17bf95ff4a50b41a9a0b9b2f</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M56" t="inlineStr">
         <is>
           <t>L19066036</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P34" t="inlineStr">
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
         <is>
           <t>1786234530</t>
         </is>
       </c>
-      <c r="S34" t="inlineStr">
+      <c r="S56" t="inlineStr">
         <is>
           <t>1786561200</t>
         </is>
       </c>
-      <c r="T34" t="inlineStr">
+      <c r="T56" t="inlineStr">
         <is>
           <t>1.830664</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr">
+      <c r="U56" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V34" t="inlineStr">
+      <c r="V56" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>